<commit_message>
Excel bijgewerkt: bol-link 42223 staat nu goed in de lijst
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lego Lijst.xlsx
+++ b/Lego Lijst.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="192">
   <si>
     <t>Bouwnummer:</t>
   </si>
@@ -571,6 +571,9 @@
   </si>
   <si>
     <t>https://www.lego.com/nl-nl/product/1966-ford-gt40-mkii-race-car-42223</t>
+  </si>
+  <si>
+    <t>https://partner.bol.com/click/click?p=2&amp;t=url&amp;s=1544332&amp;f=TXL&amp;url=https%3A%2F%2Fwww.bol.com%2Fnl%2Fnl%2Fp%2Flego-technic-1966-ford-gt40-mkii-racewagen-42223%2F9300000237345417%2F&amp;name=LEGO%20Technic%201966%20Ford%20GT40%20MKII%20Racewagen%20-%20Vintage%20Auto%20Bouwpakket%20voor%20Volwassenen...</t>
   </si>
   <si>
     <t>https://link.amazon/B0bsw6Wki</t>
@@ -592,7 +595,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -658,11 +661,6 @@
       <color rgb="FF212529"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12.0"/>
-      <color rgb="FF636363"/>
-      <name val="&quot;Cera Pro&quot;"/>
     </font>
     <font>
       <u/>
@@ -761,14 +759,14 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -3277,10 +3275,10 @@
         <v>14</v>
       </c>
       <c r="I68" s="26" t="s">
-        <v>172</v>
+        <v>186</v>
       </c>
       <c r="J68" s="26" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K68" s="2"/>
       <c r="L68" s="2"/>
@@ -3291,10 +3289,10 @@
         <v>40820.0</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C69" s="24" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D69" s="25"/>
       <c r="E69" s="2" t="s">
@@ -3310,10 +3308,10 @@
         <v>14</v>
       </c>
       <c r="I69" s="12" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J69" s="12" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K69" s="2"/>
       <c r="L69" s="2"/>

</xml_diff>

<commit_message>
Voeg set 11381 toe (Jaguar E-Type, Icons)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lego Lijst.xlsx
+++ b/Lego Lijst.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="195">
   <si>
     <t>Bouwnummer:</t>
   </si>
@@ -589,6 +589,15 @@
   </si>
   <si>
     <t>https://link.amazon/B06DhUv13</t>
+  </si>
+  <si>
+    <t>https://www.lego.com/nl-nl/product/jaguar-e-type-11381</t>
+  </si>
+  <si>
+    <t>https://partner.bol.com/click/click?p=2&amp;t=url&amp;s=1544332&amp;f=TXL&amp;url=https%3A%2F%2Fwww.bol.com%2Fnl%2Fnl%2Fp%2Flego-icons-jaguar-e-type-klassieke-sportwagen-auto-11381%2F9300000265639999%2F&amp;name=LEGO%20Icons%20Jaguar%20E-Type%20-%20Klassieke%20Sportwagen%20Auto%20-%2011381</t>
+  </si>
+  <si>
+    <t>https://link.amazon/B0g01DC7g</t>
   </si>
 </sst>
 </file>
@@ -3318,16 +3327,34 @@
       <c r="M69" s="13"/>
     </row>
     <row r="70">
-      <c r="A70" s="25"/>
-      <c r="B70" s="25"/>
-      <c r="C70" s="25"/>
+      <c r="A70" s="20">
+        <v>11381.0</v>
+      </c>
+      <c r="B70" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="C70" s="24" t="s">
+        <v>192</v>
+      </c>
       <c r="D70" s="25"/>
-      <c r="E70" s="25"/>
-      <c r="F70" s="2"/>
-      <c r="G70" s="2"/>
-      <c r="H70" s="2"/>
-      <c r="I70" s="2"/>
-      <c r="J70" s="2"/>
+      <c r="E70" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I70" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="J70" s="12" t="s">
+        <v>194</v>
+      </c>
       <c r="K70" s="2"/>
       <c r="L70" s="2"/>
       <c r="M70" s="13"/>
@@ -17584,7 +17611,10 @@
     <hyperlink r:id="rId162" ref="C69"/>
     <hyperlink r:id="rId163" ref="I69"/>
     <hyperlink r:id="rId164" ref="J69"/>
+    <hyperlink r:id="rId165" ref="C70"/>
+    <hyperlink r:id="rId166" ref="I70"/>
+    <hyperlink r:id="rId167" ref="J70"/>
   </hyperlinks>
-  <drawing r:id="rId165"/>
+  <drawing r:id="rId168"/>
 </worksheet>
 </file>
</xml_diff>